<commit_message>
fix(member-1): complete all deliverables, synchronize test cases to 132, enhance agent skill G9.5, add screenshots and export PDFs
</commit_message>
<xml_diff>
--- a/test-cases/member-1.xlsx
+++ b/test-cases/member-1.xlsx
@@ -541,7 +541,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -590,7 +589,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -3953,7 +3951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -4881,95 +4879,99 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>FR07_EXT_01</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Domain (State Transition)</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Xem giỏ hàng ngay sau khi khởi tạo tài khoản</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>User mới</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>GET /api/cart</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>Authorization: Bearer &lt;user_token&gt;</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr"/>
-      <c r="H14" s="6" t="n">
-        <v>200</v>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>200 OK + []</t>
-        </is>
-      </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>200 OK + []</t>
-        </is>
-      </c>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>Human Extension</t>
-        </is>
-      </c>
-      <c r="M14" s="12" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="N14" s="11" t="inlineStr">
-        <is>
-          <t>AI bỏ sót xác thực mảng rỗng ban đầu</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC_FR07_DOM_13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Domain Invalid</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Thêm sản phẩm với số lượng số thực không nguyên (quantity = 1.5)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>User đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>POST /api/cart</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer &lt;user_token&gt;, Content-Type: application/json</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>{"id":1,"name":"iPhone 15","price":30000000,"quantity":1.5}</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>400</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>{"error":"Số lượng sản phẩm phải là số nguyên dương"}</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK (SUT không kiểm tra số nguyên)</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>AI Baseline</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Khớp đặc tả validation</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_01</t>
+          <t>FR07_EXT_01</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>State Transition</t>
+          <t>Domain (State Transition)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Thêm 1 item vào giỏ -&gt; Giỏ chuyển từ rỗng sang có 1 item</t>
+          <t>Xem giỏ hàng ngay sau khi khởi tạo tài khoản</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Giỏ rỗng</t>
+          <t>User mới</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>POST /api/cart</t>
+          <t>GET /api/cart</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
@@ -4977,22 +4979,18 @@
           <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>{"id":1,"quantity":1}</t>
-        </is>
-      </c>
+      <c r="G15" s="11" t="inlineStr"/>
       <c r="H15" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có 1 phần tử</t>
+          <t>200 OK + []</t>
         </is>
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có 1 phần tử</t>
+          <t>200 OK + []</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -5002,7 +5000,7 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>AI Baseline</t>
+          <t>Human Extension</t>
         </is>
       </c>
       <c r="M15" s="12" t="inlineStr">
@@ -5012,14 +5010,14 @@
       </c>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>Chuyển trạng thái giỏ</t>
+          <t>AI bỏ sót xác thực mảng rỗng ban đầu</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_02</t>
+          <t>TC_FR07_ST_01</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -5029,12 +5027,12 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Thêm tiếp item thứ 2 khác loại -&gt; Giỏ có 2 items</t>
+          <t>Thêm 1 item vào giỏ -&gt; Giỏ chuyển từ rỗng sang có 1 item</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có 1 item</t>
+          <t>Giỏ rỗng</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -5049,7 +5047,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>{"id":2,"quantity":1}</t>
+          <t>{"id":1,"quantity":1}</t>
         </is>
       </c>
       <c r="H16" s="6" t="n">
@@ -5057,12 +5055,12 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có 2 phần tử</t>
+          <t>Giỏ có 1 phần tử</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có 2 phần tử</t>
+          <t>Giỏ có 1 phần tử</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -5082,14 +5080,14 @@
       </c>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>Nhiều item khác nhau</t>
+          <t>Chuyển trạng thái giỏ</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_03</t>
+          <t>TC_FR07_ST_02</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -5099,12 +5097,12 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Thêm trùng item đã có -&gt; Tự động cộng dồn số lượng</t>
+          <t>Thêm tiếp item thứ 2 khác loại -&gt; Giỏ có 2 items</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Giỏ đã có item 1</t>
+          <t>Giỏ có 1 item</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -5119,7 +5117,7 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>{"id":1,"quantity":2}</t>
+          <t>{"id":2,"quantity":1}</t>
         </is>
       </c>
       <c r="H17" s="6" t="n">
@@ -5127,17 +5125,17 @@
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>Item 1 có quantity = 3</t>
+          <t>Giỏ có 2 phần tử</t>
         </is>
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>SUT append 2 dòng riêng</t>
-        </is>
-      </c>
-      <c r="K17" s="13" t="inlineStr">
-        <is>
-          <t>FAIL (Bug Logged)</t>
+          <t>Giỏ có 2 phần tử</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -5145,21 +5143,21 @@
           <t>AI Baseline</t>
         </is>
       </c>
-      <c r="M17" s="14" t="inlineStr">
-        <is>
-          <t>INCOMPLETE</t>
+      <c r="M17" s="12" t="inlineStr">
+        <is>
+          <t>VALID</t>
         </is>
       </c>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>SUT không cộng dồn quantity</t>
+          <t>Nhiều item khác nhau</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_04</t>
+          <t>TC_FR07_ST_03</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -5169,17 +5167,17 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Cập nhật số lượng item qua PUT /api/cart</t>
+          <t>Thêm trùng item đã có -&gt; Tự động cộng dồn số lượng</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có item</t>
+          <t>Giỏ đã có item 1</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>PUT /api/cart</t>
+          <t>POST /api/cart</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -5189,7 +5187,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>{"id":1,"quantity":5}</t>
+          <t>{"id":1,"quantity":2}</t>
         </is>
       </c>
       <c r="H18" s="6" t="n">
@@ -5197,12 +5195,12 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Cập nhật thành công</t>
+          <t>Item 1 có quantity = 3</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>404 Not Found (Thiếu API)</t>
+          <t>SUT append 2 dòng riêng</t>
         </is>
       </c>
       <c r="K18" s="13" t="inlineStr">
@@ -5215,21 +5213,21 @@
           <t>AI Baseline</t>
         </is>
       </c>
-      <c r="M18" s="13" t="inlineStr">
-        <is>
-          <t>INVALID</t>
+      <c r="M18" s="14" t="inlineStr">
+        <is>
+          <t>INCOMPLETE</t>
         </is>
       </c>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>SUT chưa triển khai PUT /api/cart</t>
+          <t>SUT không cộng dồn quantity</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_05</t>
+          <t>TC_FR07_ST_04</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -5239,17 +5237,17 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Xóa 1 item khỏi giỏ qua DELETE /api/cart/1</t>
+          <t>Cập nhật số lượng item qua PUT /api/cart</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có item 1</t>
+          <t>Giỏ có item</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>DELETE /api/cart/1</t>
+          <t>PUT /api/cart</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -5257,13 +5255,17 @@
           <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr"/>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>{"id":1,"quantity":5}</t>
+        </is>
+      </c>
       <c r="H19" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>Xóa item thành công</t>
+          <t>Cập nhật thành công</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr">
@@ -5288,14 +5290,14 @@
       </c>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>SUT chưa triển khai DELETE /api/cart/:id</t>
+          <t>SUT chưa triển khai PUT /api/cart</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_06</t>
+          <t>TC_FR07_ST_05</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -5305,17 +5307,17 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Checkout giỏ hàng thành công -&gt; Chuyển sang Order</t>
+          <t>Xóa 1 item khỏi giỏ qua DELETE /api/cart/1</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có item</t>
+          <t>Giỏ có item 1</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>POST /api/checkout</t>
+          <t>DELETE /api/cart/1</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
@@ -5323,27 +5325,23 @@
           <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>{"total_amount":30000000,"shipping_address":"TP.HCM"}</t>
-        </is>
-      </c>
+      <c r="G20" s="11" t="inlineStr"/>
       <c r="H20" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>{"message":"Checkout successful"}</t>
+          <t>Xóa item thành công</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>200 OK</t>
-        </is>
-      </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>404 Not Found (Thiếu API)</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>FAIL (Bug Logged)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -5351,21 +5349,21 @@
           <t>AI Baseline</t>
         </is>
       </c>
-      <c r="M20" s="12" t="inlineStr">
-        <is>
-          <t>VALID</t>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t>INVALID</t>
         </is>
       </c>
       <c r="N20" s="11" t="inlineStr">
         <is>
-          <t>Quy trình đặt hàng</t>
+          <t>SUT chưa triển khai DELETE /api/cart/:id</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_07</t>
+          <t>TC_FR07_ST_06</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
@@ -5375,17 +5373,17 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Kiểm tra giỏ hàng sau khi checkout</t>
+          <t>Checkout giỏ hàng thành công -&gt; Chuyển sang Order</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Đã checkout</t>
+          <t>Giỏ có item</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>GET /api/cart</t>
+          <t>POST /api/checkout</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
@@ -5393,18 +5391,22 @@
           <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr"/>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>{"total_amount":30000000,"shipping_address":"TP.HCM"}</t>
+        </is>
+      </c>
       <c r="H21" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>Giỏ hàng reset</t>
+          <t>{"message":"Checkout successful"}</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>Giỏ vẫn giữ nguyên</t>
+          <t>200 OK</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -5424,14 +5426,14 @@
       </c>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>Chu trình thanh toán</t>
+          <t>Quy trình đặt hàng</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_08</t>
+          <t>TC_FR07_ST_07</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -5441,12 +5443,12 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Kiểm tra tính bền vững dữ liệu giỏ khi server restart</t>
+          <t>Kiểm tra giỏ hàng sau khi checkout</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Giỏ có item</t>
+          <t>Đã checkout</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -5465,12 +5467,12 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Giỏ giữ nguyên</t>
+          <t>Giỏ hàng reset</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>Mất trắng dữ liệu (In-memory)</t>
+          <t>Giỏ vẫn giữ nguyên</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
@@ -5483,21 +5485,21 @@
           <t>AI Baseline</t>
         </is>
       </c>
-      <c r="M22" s="14" t="inlineStr">
-        <is>
-          <t>INCOMPLETE</t>
+      <c r="M22" s="12" t="inlineStr">
+        <is>
+          <t>VALID</t>
         </is>
       </c>
       <c r="N22" s="11" t="inlineStr">
         <is>
-          <t>SUT lưu in-memory userCarts</t>
+          <t>Chu trình thanh toán</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_ST_09</t>
+          <t>TC_FR07_ST_08</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -5507,12 +5509,12 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Đăng xuất và đăng nhập lại vẫn thấy giỏ hàng</t>
+          <t>Kiểm tra tính bền vững dữ liệu giỏ khi server restart</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>User login lại</t>
+          <t>Giỏ có item</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -5531,12 +5533,12 @@
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>Giỏ hàng tồn tại</t>
+          <t>Giỏ giữ nguyên</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>Giỏ hàng tồn tại</t>
+          <t>Mất trắng dữ liệu (In-memory)</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -5549,36 +5551,36 @@
           <t>AI Baseline</t>
         </is>
       </c>
-      <c r="M23" s="12" t="inlineStr">
-        <is>
-          <t>VALID</t>
+      <c r="M23" s="14" t="inlineStr">
+        <is>
+          <t>INCOMPLETE</t>
         </is>
       </c>
       <c r="N23" s="11" t="inlineStr">
         <is>
-          <t>Tính liên tục phiên</t>
+          <t>SUT lưu in-memory userCarts</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>FR07_EXT_02</t>
+          <t>TC_FR07_ST_09</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>State (Multi-tenant)</t>
+          <t>State Transition</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>User A thêm giỏ, User B đăng nhập xem giỏ đảm bảo cô lập</t>
+          <t>Đăng xuất và đăng nhập lại vẫn thấy giỏ hàng</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>User A và B riêng biệt</t>
+          <t>User login lại</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -5588,7 +5590,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;userB_token&gt;</t>
+          <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr"/>
@@ -5597,12 +5599,12 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Giỏ User B rỗng</t>
+          <t>Giỏ hàng tồn tại</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>Giỏ User B rỗng</t>
+          <t>Giỏ hàng tồn tại</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
@@ -5612,7 +5614,7 @@
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>Human Extension</t>
+          <t>AI Baseline</t>
         </is>
       </c>
       <c r="M24" s="12" t="inlineStr">
@@ -5622,57 +5624,53 @@
       </c>
       <c r="N24" s="11" t="inlineStr">
         <is>
-          <t>AI bỏ sót xác thực cô lập đa người dùng</t>
+          <t>Tính liên tục phiên</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>FR07_EXT_03</t>
+          <t>FR07_EXT_02</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>State (Quantity Coercion)</t>
+          <t>State (Multi-tenant)</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Thêm sản phẩm với quantity dạng chuỗi '2'</t>
+          <t>User A thêm giỏ, User B đăng nhập xem giỏ đảm bảo cô lập</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>User đăng nhập</t>
+          <t>User A và B riêng biệt</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>POST /api/cart</t>
+          <t>GET /api/cart</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;user_token&gt;</t>
-        </is>
-      </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>{"id":1,"quantity":"2"}</t>
-        </is>
-      </c>
+          <t>Authorization: Bearer &lt;userB_token&gt;</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr"/>
       <c r="H25" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>200 OK + ép kiểu int</t>
+          <t>Giỏ User B rỗng</t>
         </is>
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>200 OK</t>
+          <t>Giỏ User B rỗng</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -5692,49 +5690,57 @@
       </c>
       <c r="N25" s="11" t="inlineStr">
         <is>
-          <t>AI bỏ sót kiểm tra ép kiểu quantity</t>
+          <t>AI bỏ sót xác thực cô lập đa người dùng</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_01</t>
+          <t>FR07_EXT_03</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Security (No Auth)</t>
+          <t>State (Quantity Coercion)</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Xem giỏ hàng không truyền Authorization header</t>
+          <t>Thêm sản phẩm với quantity dạng chuỗi '2'</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Không token</t>
+          <t>User đăng nhập</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>GET /api/cart</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr"/>
-      <c r="G26" s="11" t="inlineStr"/>
+          <t>POST /api/cart</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer &lt;user_token&gt;</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>{"id":1,"quantity":"2"}</t>
+        </is>
+      </c>
       <c r="H26" s="6" t="n">
-        <v>401</v>
+        <v>200</v>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>{"error":"Unauthorized"}</t>
+          <t>200 OK + ép kiểu int</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr">
         <is>
-          <t>401 Unauthorized</t>
+          <t>200 OK</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
@@ -5744,7 +5750,7 @@
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>AI Baseline</t>
+          <t>Human Extension</t>
         </is>
       </c>
       <c r="M26" s="12" t="inlineStr">
@@ -5754,14 +5760,14 @@
       </c>
       <c r="N26" s="11" t="inlineStr">
         <is>
-          <t>Bắt buộc token xác thực</t>
+          <t>AI bỏ sót kiểm tra ép kiểu quantity</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_02</t>
+          <t>TC_FR07_SEC_01</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -5771,7 +5777,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Thêm giỏ hàng không truyền Authorization header</t>
+          <t>Xem giỏ hàng không truyền Authorization header</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -5781,15 +5787,11 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>POST /api/cart</t>
+          <t>GET /api/cart</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr"/>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>{"id":1,"quantity":1}</t>
-        </is>
-      </c>
+      <c r="G27" s="11" t="inlineStr"/>
       <c r="H27" s="6" t="n">
         <v>401</v>
       </c>
@@ -5820,53 +5822,53 @@
       </c>
       <c r="N27" s="11" t="inlineStr">
         <is>
-          <t>Bắt buộc token khi thêm giỏ</t>
+          <t>Bắt buộc token xác thực</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_03</t>
+          <t>TC_FR07_SEC_02</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Security (Invalid Token)</t>
+          <t>Security (No Auth)</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Gửi request với JWT Token sai chữ ký</t>
+          <t>Thêm giỏ hàng không truyền Authorization header</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Token giả</t>
+          <t>Không token</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>GET /api/cart</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr">
-        <is>
-          <t>Authorization: Bearer fake_token</t>
-        </is>
-      </c>
-      <c r="G28" s="11" t="inlineStr"/>
+          <t>POST /api/cart</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr"/>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>{"id":1,"quantity":1}</t>
+        </is>
+      </c>
       <c r="H28" s="6" t="n">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>{"error":"Forbidden"}</t>
+          <t>{"error":"Unauthorized"}</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
-          <t>403 Forbidden</t>
+          <t>401 Unauthorized</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
@@ -5886,53 +5888,53 @@
       </c>
       <c r="N28" s="11" t="inlineStr">
         <is>
-          <t>Từ chối token giả</t>
+          <t>Bắt buộc token khi thêm giỏ</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_04</t>
+          <t>TC_FR07_SEC_03</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Security (IDOR)</t>
+          <t>Security (Invalid Token)</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>User A cố gắng xem giỏ hàng của User B</t>
+          <t>Gửi request với JWT Token sai chữ ký</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>User A token</t>
+          <t>Token giả</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>GET /api/cart?user_id=2</t>
+          <t>GET /api/cart</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;userA_token&gt;</t>
+          <t>Authorization: Bearer fake_token</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr"/>
       <c r="H29" s="6" t="n">
-        <v>200</v>
+        <v>403</v>
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>Chỉ thấy giỏ User A</t>
+          <t>{"error":"Forbidden"}</t>
         </is>
       </c>
       <c r="J29" s="11" t="inlineStr">
         <is>
-          <t>Chỉ thấy giỏ User A</t>
+          <t>403 Forbidden</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -5952,57 +5954,53 @@
       </c>
       <c r="N29" s="11" t="inlineStr">
         <is>
-          <t>Chống IDOR qua query param</t>
+          <t>Từ chối token giả</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_05</t>
+          <t>TC_FR07_SEC_04</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Security (SQLi)</t>
+          <t>Security (IDOR)</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>SQLi trong trường name sản phẩm thêm vào giỏ</t>
+          <t>User A cố gắng xem giỏ hàng của User B</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>User đăng nhập</t>
+          <t>User A token</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>POST /api/cart</t>
+          <t>GET /api/cart?user_id=2</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;user_token&gt;</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>{"id":1,"name":"' OR 1=1 --","quantity":1}</t>
-        </is>
-      </c>
+          <t>Authorization: Bearer &lt;userA_token&gt;</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr"/>
       <c r="H30" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Lưu an toàn dạng chuỗi</t>
+          <t>Chỉ thấy giỏ User A</t>
         </is>
       </c>
       <c r="J30" s="11" t="inlineStr">
         <is>
-          <t>Lưu an toàn</t>
+          <t>Chỉ thấy giỏ User A</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
@@ -6022,24 +6020,24 @@
       </c>
       <c r="N30" s="11" t="inlineStr">
         <is>
-          <t>Chống SQLi payload</t>
+          <t>Chống IDOR qua query param</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_06</t>
+          <t>TC_FR07_SEC_05</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Security (Tampered Price)</t>
+          <t>Security (SQLi)</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Client tự truyền giá price = 1đ vào giỏ hàng</t>
+          <t>SQLi trong trường name sản phẩm thêm vào giỏ</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
@@ -6059,25 +6057,25 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>{"id":1,"price":1,"quantity":1}</t>
+          <t>{"id":1,"name":"' OR 1=1 --","quantity":1}</t>
         </is>
       </c>
       <c r="H31" s="6" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
-          <t>Backend phải lấy giá từ CSDL</t>
+          <t>Lưu an toàn dạng chuỗi</t>
         </is>
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>SUT lưu giá 1đ từ client</t>
-        </is>
-      </c>
-      <c r="K31" s="13" t="inlineStr">
-        <is>
-          <t>FAIL (Bug Logged)</t>
+          <t>Lưu an toàn</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -6085,31 +6083,31 @@
           <t>AI Baseline</t>
         </is>
       </c>
-      <c r="M31" s="14" t="inlineStr">
-        <is>
-          <t>INCOMPLETE</t>
+      <c r="M31" s="12" t="inlineStr">
+        <is>
+          <t>VALID</t>
         </is>
       </c>
       <c r="N31" s="11" t="inlineStr">
         <is>
-          <t>SUT dính lỗ hổng Price Tampering</t>
+          <t>Chống SQLi payload</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_07</t>
+          <t>TC_FR07_SEC_06</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Security (XSS)</t>
+          <t>Security (Tampered Price)</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>XSS payload trong trường ghi chú sản phẩm</t>
+          <t>Client tự truyền giá price = 1đ vào giỏ hàng</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -6129,25 +6127,25 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>{"id":1,"note":"&lt;script&gt;alert(1)&lt;/script&gt;"}</t>
+          <t>{"id":1,"price":1,"quantity":1}</t>
         </is>
       </c>
       <c r="H32" s="6" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Không thực thi script</t>
+          <t>Backend phải lấy giá từ CSDL</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
-          <t>Lưu chuỗi an toàn</t>
-        </is>
-      </c>
-      <c r="K32" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>SUT lưu giá 1đ từ client</t>
+        </is>
+      </c>
+      <c r="K32" s="13" t="inlineStr">
+        <is>
+          <t>FAIL (Bug Logged)</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
@@ -6155,60 +6153,64 @@
           <t>AI Baseline</t>
         </is>
       </c>
-      <c r="M32" s="12" t="inlineStr">
-        <is>
-          <t>VALID</t>
+      <c r="M32" s="14" t="inlineStr">
+        <is>
+          <t>INCOMPLETE</t>
         </is>
       </c>
       <c r="N32" s="11" t="inlineStr">
         <is>
-          <t>Chống XSS giỏ hàng</t>
+          <t>SUT dính lỗ hổng Price Tampering</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_08</t>
+          <t>TC_FR07_SEC_07</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Security (Admin Access)</t>
+          <t>Security (XSS)</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Admin xem giỏ hàng cá nhân không bị trộn với khách</t>
+          <t>XSS payload trong trường ghi chú sản phẩm</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Admin token</t>
+          <t>User đăng nhập</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>GET /api/cart</t>
+          <t>POST /api/cart</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;admin_token&gt;</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="inlineStr"/>
+          <t>Authorization: Bearer &lt;user_token&gt;</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>{"id":1,"note":"&lt;script&gt;alert(1)&lt;/script&gt;"}</t>
+        </is>
+      </c>
       <c r="H33" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>Giỏ hàng admin riêng</t>
+          <t>Không thực thi script</t>
         </is>
       </c>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>Giỏ hàng riêng biệt</t>
+          <t>Lưu chuỗi an toàn</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -6228,29 +6230,29 @@
       </c>
       <c r="N33" s="11" t="inlineStr">
         <is>
-          <t>Phân quyền theo userId</t>
+          <t>Chống XSS giỏ hàng</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SEC_09</t>
+          <t>TC_FR07_SEC_08</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Security (Expired Token)</t>
+          <t>Security (Admin Access)</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Gửi request với token đã hết hạn</t>
+          <t>Admin xem giỏ hàng cá nhân không bị trộn với khách</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Token hết hạn</t>
+          <t>Admin token</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -6260,21 +6262,21 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;expired_token&gt;</t>
+          <t>Authorization: Bearer &lt;admin_token&gt;</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr"/>
       <c r="H34" s="6" t="n">
-        <v>403</v>
+        <v>200</v>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>{"error":"Forbidden"}</t>
+          <t>Giỏ hàng admin riêng</t>
         </is>
       </c>
       <c r="J34" s="11" t="inlineStr">
         <is>
-          <t>403 Forbidden</t>
+          <t>Giỏ hàng riêng biệt</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
@@ -6294,29 +6296,29 @@
       </c>
       <c r="N34" s="11" t="inlineStr">
         <is>
-          <t>Kiểm tra hạn sử dụng token</t>
+          <t>Phân quyền theo userId</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>FR07_EXT_04</t>
+          <t>TC_FR07_SEC_09</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Security (Header Tampering)</t>
+          <t>Security (Expired Token)</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Gửi token với prefix sai 'Token &lt;jwt&gt;' thay vì 'Bearer &lt;jwt&gt;'</t>
+          <t>Gửi request với token đã hết hạn</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>User token</t>
+          <t>Token hết hạn</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -6326,21 +6328,21 @@
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Token &lt;user_token&gt;</t>
+          <t>Authorization: Bearer &lt;expired_token&gt;</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr"/>
       <c r="H35" s="6" t="n">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>401 Unauthorized</t>
+          <t>{"error":"Forbidden"}</t>
         </is>
       </c>
       <c r="J35" s="11" t="inlineStr">
         <is>
-          <t>401 Unauthorized</t>
+          <t>403 Forbidden</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -6350,7 +6352,7 @@
       </c>
       <c r="L35" s="6" t="inlineStr">
         <is>
-          <t>Human Extension</t>
+          <t>AI Baseline</t>
         </is>
       </c>
       <c r="M35" s="12" t="inlineStr">
@@ -6360,29 +6362,29 @@
       </c>
       <c r="N35" s="11" t="inlineStr">
         <is>
-          <t>AI bỏ sót định dạng chuẩn Bearer</t>
+          <t>Kiểm tra hạn sử dụng token</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>FR07_EXT_05</t>
+          <t>FR07_EXT_04</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Security (Empty Bearer)</t>
+          <t>Security (Header Tampering)</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Gửi header Authorization: Bearer để trống token</t>
+          <t>Gửi token với prefix sai 'Token &lt;jwt&gt;' thay vì 'Bearer &lt;jwt&gt;'</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Token rỗng</t>
+          <t>User token</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -6392,7 +6394,7 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Authorization: Bearer </t>
+          <t>Authorization: Token &lt;user_token&gt;</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr"/>
@@ -6426,29 +6428,29 @@
       </c>
       <c r="N36" s="11" t="inlineStr">
         <is>
-          <t>AI bỏ sót trường hợp Bearer rỗng</t>
+          <t>AI bỏ sót định dạng chuẩn Bearer</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SCH_01</t>
+          <t>FR07_EXT_05</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Schema Validation</t>
+          <t>Security (Empty Bearer)</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Validate JSON Schema GET /api/cart (Mảng các CartItem)</t>
+          <t>Gửi header Authorization: Bearer để trống token</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>User đăng nhập</t>
+          <t>Token rỗng</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -6458,21 +6460,21 @@
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;user_token&gt;</t>
+          <t xml:space="preserve">Authorization: Bearer </t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr"/>
       <c r="H37" s="6" t="n">
-        <v>200</v>
+        <v>401</v>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>Khớp Cart Array Schema</t>
+          <t>401 Unauthorized</t>
         </is>
       </c>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>Khớp schema 100%</t>
+          <t>401 Unauthorized</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
@@ -6482,7 +6484,7 @@
       </c>
       <c r="L37" s="6" t="inlineStr">
         <is>
-          <t>AI Baseline</t>
+          <t>Human Extension</t>
         </is>
       </c>
       <c r="M37" s="12" t="inlineStr">
@@ -6492,14 +6494,14 @@
       </c>
       <c r="N37" s="11" t="inlineStr">
         <is>
-          <t>Schema mảng giỏ hàng</t>
+          <t>AI bỏ sót trường hợp Bearer rỗng</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SCH_02</t>
+          <t>TC_FR07_SCH_01</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -6509,7 +6511,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Validate JSON Schema POST /api/cart ({message: string})</t>
+          <t>Validate JSON Schema GET /api/cart (Mảng các CartItem)</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -6519,7 +6521,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>POST /api/cart</t>
+          <t>GET /api/cart</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -6527,17 +6529,13 @@
           <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr">
-        <is>
-          <t>{"id":3,"quantity":1}</t>
-        </is>
-      </c>
+      <c r="G38" s="11" t="inlineStr"/>
       <c r="H38" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Khớp POST Cart Schema</t>
+          <t>Khớp Cart Array Schema</t>
         </is>
       </c>
       <c r="J38" s="11" t="inlineStr">
@@ -6562,14 +6560,14 @@
       </c>
       <c r="N38" s="11" t="inlineStr">
         <is>
-          <t>Schema response thêm giỏ</t>
+          <t>Schema mảng giỏ hàng</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SCH_03</t>
+          <t>TC_FR07_SCH_02</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
@@ -6579,32 +6577,40 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Validate JSON Schema lỗi 401 khi thiếu token</t>
+          <t>Validate JSON Schema POST /api/cart ({message: string})</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Không token</t>
+          <t>User đăng nhập</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>GET /api/cart</t>
-        </is>
-      </c>
-      <c r="F39" s="11" t="inlineStr"/>
-      <c r="G39" s="11" t="inlineStr"/>
+          <t>POST /api/cart</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer &lt;user_token&gt;</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>{"id":3,"quantity":1}</t>
+        </is>
+      </c>
       <c r="H39" s="6" t="n">
-        <v>401</v>
+        <v>200</v>
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>Khớp Error Schema {error: string}</t>
+          <t>Khớp POST Cart Schema</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>Khớp schema error</t>
+          <t>Khớp schema 100%</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
@@ -6624,14 +6630,14 @@
       </c>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>Schema lỗi 401</t>
+          <t>Schema response thêm giỏ</t>
         </is>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SCH_04</t>
+          <t>TC_FR07_SCH_03</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -6641,12 +6647,12 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Validate JSON Schema lỗi 403 khi token không hợp lệ</t>
+          <t>Validate JSON Schema lỗi 401 khi thiếu token</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Token giả</t>
+          <t>Không token</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
@@ -6654,14 +6660,10 @@
           <t>GET /api/cart</t>
         </is>
       </c>
-      <c r="F40" s="11" t="inlineStr">
-        <is>
-          <t>Authorization: Bearer fake</t>
-        </is>
-      </c>
+      <c r="F40" s="11" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr"/>
       <c r="H40" s="6" t="n">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
@@ -6690,14 +6692,14 @@
       </c>
       <c r="N40" s="11" t="inlineStr">
         <is>
-          <t>Schema lỗi 403</t>
+          <t>Schema lỗi 401</t>
         </is>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SCH_05</t>
+          <t>TC_FR07_SCH_04</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
@@ -6707,12 +6709,12 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Header Content-Type của GET /api/cart là application/json</t>
+          <t>Validate JSON Schema lỗi 403 khi token không hợp lệ</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>User đăng nhập</t>
+          <t>Token giả</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
@@ -6722,21 +6724,21 @@
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Authorization: Bearer &lt;user_token&gt;</t>
+          <t>Authorization: Bearer fake</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr"/>
       <c r="H41" s="6" t="n">
-        <v>200</v>
+        <v>403</v>
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>Content-Type: application/json</t>
+          <t>Khớp Error Schema {error: string}</t>
         </is>
       </c>
       <c r="J41" s="11" t="inlineStr">
         <is>
-          <t>Header hợp lệ</t>
+          <t>Khớp schema error</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
@@ -6756,14 +6758,14 @@
       </c>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>Kiểm tra content-type</t>
+          <t>Schema lỗi 403</t>
         </is>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SCH_06</t>
+          <t>TC_FR07_SCH_05</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -6773,7 +6775,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Mỗi CartItem trong mảng phải có đủ: id, quantity</t>
+          <t>Header Content-Type của GET /api/cart là application/json</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -6797,12 +6799,12 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Từng item đủ trường</t>
+          <t>Content-Type: application/json</t>
         </is>
       </c>
       <c r="J42" s="11" t="inlineStr">
         <is>
-          <t>Đủ trường bắt buộc</t>
+          <t>Header hợp lệ</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr">
@@ -6822,14 +6824,14 @@
       </c>
       <c r="N42" s="11" t="inlineStr">
         <is>
-          <t>Kiểm tra item schema</t>
+          <t>Kiểm tra content-type</t>
         </is>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>TC_FR07_SCH_07</t>
+          <t>TC_FR07_SCH_06</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
@@ -6839,7 +6841,7 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Validate Response POST /api/cart rỗng body {}</t>
+          <t>Mỗi CartItem trong mảng phải có đủ: id, quantity</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
@@ -6849,7 +6851,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>POST /api/cart</t>
+          <t>GET /api/cart</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
@@ -6857,22 +6859,18 @@
           <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
+      <c r="G43" s="11" t="inlineStr"/>
       <c r="H43" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>Xử lý body rỗng</t>
+          <t>Từng item đủ trường</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>200 OK</t>
+          <t>Đủ trường bắt buộc</t>
         </is>
       </c>
       <c r="K43" s="7" t="inlineStr">
@@ -6892,24 +6890,24 @@
       </c>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>Body rỗng</t>
+          <t>Kiểm tra item schema</t>
         </is>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>FR07_EXT_06</t>
+          <t>TC_FR07_SCH_07</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Performance / Latency</t>
+          <t>Schema Validation</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Thời gian phản hồi GET /api/cart dưới 500ms</t>
+          <t>Validate Response POST /api/cart rỗng body {}</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -6919,7 +6917,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>GET /api/cart</t>
+          <t>POST /api/cart</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
@@ -6927,36 +6925,106 @@
           <t>Authorization: Bearer &lt;user_token&gt;</t>
         </is>
       </c>
-      <c r="G44" s="11" t="inlineStr"/>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
       <c r="H44" s="6" t="n">
         <v>200</v>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
+          <t>Xử lý body rỗng</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>AI Baseline</t>
+        </is>
+      </c>
+      <c r="M44" s="12" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="N44" s="11" t="inlineStr">
+        <is>
+          <t>Body rỗng</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>FR07_EXT_06</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>Performance / Latency</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>Thời gian phản hồi GET /api/cart dưới 500ms</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>User đăng nhập</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>GET /api/cart</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer &lt;user_token&gt;</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr"/>
+      <c r="H45" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
           <t>responseTime &lt; 500ms</t>
         </is>
       </c>
-      <c r="J44" s="11" t="inlineStr">
+      <c r="J45" s="11" t="inlineStr">
         <is>
           <t>Response time: 2ms</t>
         </is>
       </c>
-      <c r="K44" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L44" s="6" t="inlineStr">
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="inlineStr">
         <is>
           <t>Human Extension</t>
         </is>
       </c>
-      <c r="M44" s="12" t="inlineStr">
-        <is>
-          <t>VALID</t>
-        </is>
-      </c>
-      <c r="N44" s="11" t="inlineStr">
+      <c r="M45" s="12" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="N45" s="11" t="inlineStr">
         <is>
           <t>AI bỏ sót kiểm tra hiệu năng NFR giỏ hàng</t>
         </is>

</xml_diff>